<commit_message>
VISU PTBG 2.5.1 : documentation réorganisée
- POINTS_OUVERTS.md retiré : les 18 questions sont dans le récapitulatif
  Excel (onglet « Points ouverts »), document unique à faire valider ; la
  qualification restant à faire passe à la fin de la matrice de traçabilité.
- README : point d'entrée court, tableau « quelle documentation lire ? ».
- Traçabilité : synthèse des statuts en tête.
- Guide : sommaire, tableaux (réglages, onglets, rapports, préférences),
  section 12 « Raccourcis ».
- Architecture : flux de données en tableau.
- Dépendances : « En bref », campagne 2.5.x, campagne 2.1.0 résumée.
- Compatibilité : essai de réception sous forme de fiche à remplir.
- Capture du diagnostic mise à jour. Code inchangé (deux commentaires).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xr679nCBrcWe6H8towhecz
</commit_message>
<xml_diff>
--- a/docs/recapitulatif/Recapitulatif_requis_VISU_PTBG.xlsx
+++ b/docs/recapitulatif/Recapitulatif_requis_VISU_PTBG.xlsx
@@ -39,7 +39,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1621" uniqueCount="1028">
   <si>
-    <t xml:space="preserve">Récapitulatif des requis — VISU PTBG 2.5.0</t>
+    <t xml:space="preserve">Récapitulatif des requis — VISU PTBG 2.5.1</t>
   </si>
   <si>
     <t xml:space="preserve">Spécification NCS/00/I/COMMON----/ES/010 Rev. A (13/10/2026) — relecture : Sébastien Kubasik — état au 28/10/2026</t>
@@ -7268,7 +7268,7 @@
         <v>561</v>
       </c>
       <c r="D2" s="19" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E2" s="19" t="n">
         <v>5</v>

</xml_diff>

<commit_message>
VISU PTBG 1.0.0 : première version livrée pour revue des requis
La version envoyée au rédacteur de la spécification devient la 1.0.0 : le
CHANGELOG repart d'une seule entrée (contenu de la version, ce qui reste à
qualifier) et les documents ne citent plus les versions intermédiaires de
développement. Code inchangé.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xr679nCBrcWe6H8towhecz
</commit_message>
<xml_diff>
--- a/docs/recapitulatif/Recapitulatif_requis_VISU_PTBG.xlsx
+++ b/docs/recapitulatif/Recapitulatif_requis_VISU_PTBG.xlsx
@@ -39,7 +39,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1621" uniqueCount="1028">
   <si>
-    <t xml:space="preserve">Récapitulatif des requis — VISU PTBG 2.5.1</t>
+    <t xml:space="preserve">Récapitulatif des requis — VISU PTBG 1.0.0</t>
   </si>
   <si>
     <t xml:space="preserve">Spécification NCS/00/I/COMMON----/ES/010 Rev. A (13/10/2026) — relecture : Sébastien Kubasik — état au 28/10/2026</t>
@@ -1733,7 +1733,7 @@
     <t xml:space="preserve">Que faire d'une ligne incomplète, d'un en-tête absent ou répété, d'un horodatage aberrant ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Une ligne au mauvais nombre de champs est rejetée et listée (jamais complétée : sa dernière valeur pourrait être tronquée). Sans en-tête, la 1re ligne de mesures est gardée (colonnes Colonne_1…). Un en-tête répété (fichiers concaténés) est ignoré. Un horodatage isolé à plus de 10 périodes de ses deux voisins (qui se suivent normalement) est déclaré aberrant : ERREUR, exclu du seul calcul du raster (au lieu d'un faux retour arrière suivi d'un faux trou). Depuis la 2.3.0, il reste affiché à son instant brut sur les courbes (la vue initiale est cadrée sans lui) ; case « Masquer » par fichier dans Base de temps &gt; Configurer. Valeur de 10 périodes arbitraire, réglable dans Outils &gt; Préférences (aberrant_jump_periods) : à valider. Pour une heure hh:mm:ss, une valeur isolée à plus de 12 h de ses voisins, vers l'arrière ou vers l'avant (2.2.0), n'est jamais comptée comme un passage de minuit.</t>
+    <t xml:space="preserve">Une ligne au mauvais nombre de champs est rejetée et listée (jamais complétée : sa dernière valeur pourrait être tronquée). Sans en-tête, la 1re ligne de mesures est gardée (colonnes Colonne_1…). Un en-tête répété (fichiers concaténés) est ignoré. Un horodatage isolé à plus de 10 périodes de ses deux voisins (qui se suivent normalement) est déclaré aberrant : ERREUR, exclu du seul calcul du raster (au lieu d'un faux retour arrière suivi d'un faux trou). Il reste affiché à son instant brut sur les courbes (la vue initiale est cadrée sans lui) ; case « Masquer » par fichier dans Base de temps &gt; Configurer. Valeur de 10 périodes arbitraire, réglable dans Outils &gt; Préférences (aberrant_jump_periods) : à valider. Pour une heure hh:mm:ss, une valeur isolée à plus de 12 h de ses voisins, vers l'arrière ou vers l'avant, n'est jamais comptée comme un passage de minuit.</t>
   </si>
   <si>
     <t xml:space="preserve">core/csv_reader.py, core/time_base.py (OUTLIER_JUMP), config.py (aberrant_jump_periods), core/time_parser.py (_day_offsets)</t>

</xml_diff>

<commit_message>
VISU PTBG 1.0.0 : étiquettes du graphique déplaçables à la souris
En plus des légendes des axes : légende du Time Base Monitor, noms des
pistes logiques et étiquettes des curseurs (C1, C2, Global, Δt, curseur
horizontal, point X/Y) se déplacent à la souris. Le déplacement est gardé
en fraction de la taille de l'axe (même place par rapport aux courbes à
l'écran et dans le rapport), au redessin et dans le projet ; le curseur ne
bouge pas ; un élément lâché au bord reste dans la figure. « Vue d'origine »
et le menu de l'axe (« Remettre les étiquettes à leur place ») les replacent.

145 tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xr679nCBrcWe6H8towhecz
</commit_message>
<xml_diff>
--- a/docs/recapitulatif/Recapitulatif_requis_VISU_PTBG.xlsx
+++ b/docs/recapitulatif/Recapitulatif_requis_VISU_PTBG.xlsx
@@ -25,7 +25,7 @@
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Requis!$1:$1</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Requis!$A$1:$L$65</definedName>
     <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Titles" vbProcedure="false">Tests!$1:$1</definedName>
-    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Tests!$A$1:$E$145</definedName>
+    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Tests!$A$1:$E$146</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1647" uniqueCount="1046">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1652" uniqueCount="1049">
   <si>
     <t xml:space="preserve">Récapitulatif des requis — VISU PTBG 1.0.0</t>
   </si>
@@ -132,7 +132,7 @@
     <t xml:space="preserve">Lecture des statuts :</t>
   </si>
   <si>
-    <t xml:space="preserve">• Implémenté et testé : fonction présente et associée à au moins un test automatique qui en vérifie un cas représentatif (144 tests, tous OK).</t>
+    <t xml:space="preserve">• Implémenté et testé : fonction présente et associée à au moins un test automatique qui en vérifie un cas représentatif (145 tests, tous OK).</t>
   </si>
   <si>
     <t xml:space="preserve">  Un test associé ne prouve pas à lui seul que toute l'exigence est satisfaite : la revue des énoncés avec Sébastien le confirmera.</t>
@@ -150,7 +150,7 @@
     <t xml:space="preserve">Vérifications faites le 28/10/2026 : 64 lignes du Word toutes présentes dans la matrice, chaque requis cité dans le code et dans au moins un test</t>
   </si>
   <si>
-    <t xml:space="preserve">(tools/verifier_tracabilite.py : « Traçabilité complète ») ; chaque fichier, fonction et test cité ici existe ; 144/144 tests OK (Python 3.11 de référence,</t>
+    <t xml:space="preserve">(tools/verifier_tracabilite.py : « Traçabilité complète ») ; chaque fichier, fonction et test cité ici existe ; 145/145 tests OK (Python 3.11 de référence,</t>
   </si>
   <si>
     <t xml:space="preserve">et campagne Python 3.10 à 3.14, Tk 8.6 et 9). Colonne jaune « Réponse de Sébastien » de l'onglet Points ouverts : à remplir lors de la revue.</t>
@@ -828,7 +828,8 @@
     <t xml:space="preserve">plotting/monitor.py, plotting/renderer.py</t>
   </si>
   <si>
-    <t xml:space="preserve">test_package_report.test_every_template_has_time_base_monitor</t>
+    <t xml:space="preserve">test_package_report.test_every_template_has_time_base_monitor
+test_gui.test_labels_and_monitor_legend_can_be_moved</t>
   </si>
   <si>
     <t xml:space="preserve">REQ_COMMON_KH_4103</t>
@@ -1074,7 +1075,8 @@
     <t xml:space="preserve">test_gui.test_xy_tab_and_point_pick
 test_gui.test_tabs_close_with_their_cross
 test_gui.test_reset_view_returns_to_full_duration
-test_gui.test_legend_can_be_moved_hidden_and_picks_curves</t>
+test_gui.test_legend_can_be_moved_hidden_and_picks_curves
+test_gui.test_labels_and_monitor_legend_can_be_moved</t>
   </si>
   <si>
     <t xml:space="preserve">REQ_COMMON_KH_5200</t>
@@ -1202,7 +1204,8 @@
   <si>
     <t xml:space="preserve">test_package_report.test_cursor_labels_show_time_and_value
 test_analysis_tools.test_nearest_and_hold_without_interpolation
-test_package_report.test_crowded_report_page_stays_readable</t>
+test_package_report.test_crowded_report_page_stays_readable
+test_gui.test_labels_and_monitor_legend_can_be_moved</t>
   </si>
   <si>
     <t xml:space="preserve">Implémenté — interprétation à valider (état maintenu des Bool)</t>
@@ -1405,7 +1408,8 @@
     <t xml:space="preserve">test_package_report.test_pdf_automatic_and_step_by_step
 test_package_report.test_report_page_layout_like_project_test_reports
 test_gui.test_legend_can_be_moved_hidden_and_picks_curves
-test_package_report.test_crowded_report_page_stays_readable</t>
+test_package_report.test_crowded_report_page_stays_readable
+test_gui.test_labels_and_monitor_legend_can_be_moved</t>
   </si>
   <si>
     <t xml:space="preserve">REQ_COMMON_KH_6002</t>
@@ -2655,6 +2659,15 @@
   </si>
   <si>
     <t xml:space="preserve">5406</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_labels_and_monitor_legend_can_be_moved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REQ 5106 / 5401 / 4102 / 6001 : noms des pistes logiques, étiquettes des curseurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4102, 5106, 5401, 6001</t>
   </si>
   <si>
     <t xml:space="preserve">test_dialogs_speak_french</t>
@@ -4047,8 +4060,8 @@
         <v>15</v>
       </c>
       <c r="B15" s="12" t="n">
-        <f aca="false">COUNTA(Tests!$C$2:$C$145)</f>
-        <v>144</v>
+        <f aca="false">COUNTA(Tests!$C$2:$C$146)</f>
+        <v>145</v>
       </c>
       <c r="C15" s="13"/>
     </row>
@@ -5573,7 +5586,7 @@
         <v>252</v>
       </c>
       <c r="I32" s="19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J32" s="19" t="s">
         <v>5</v>
@@ -5961,7 +5974,7 @@
       </c>
       <c r="L43" s="19"/>
     </row>
-    <row r="44" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="19" t="s">
         <v>24</v>
       </c>
@@ -5985,7 +5998,7 @@
         <v>327</v>
       </c>
       <c r="I44" s="19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J44" s="19" t="s">
         <v>5</v>
@@ -6201,7 +6214,7 @@
       </c>
       <c r="L50" s="19"/>
     </row>
-    <row r="51" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="19" t="s">
         <v>27</v>
       </c>
@@ -6225,7 +6238,7 @@
         <v>368</v>
       </c>
       <c r="I51" s="19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J51" s="19" t="s">
         <v>6</v>
@@ -6551,7 +6564,7 @@
       </c>
       <c r="L60" s="19"/>
     </row>
-    <row r="61" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="19" t="s">
         <v>29</v>
       </c>
@@ -6575,7 +6588,7 @@
         <v>433</v>
       </c>
       <c r="I61" s="19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J61" s="19" t="s">
         <v>5</v>
@@ -7348,7 +7361,7 @@
         <v>568</v>
       </c>
       <c r="D3" s="19" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E3" s="19" t="n">
         <v>13</v>
@@ -7668,10 +7681,10 @@
         <v>617</v>
       </c>
       <c r="D19" s="19" t="n">
-        <v>582</v>
+        <v>625</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F19" s="19" t="s">
         <v>618</v>
@@ -7688,7 +7701,7 @@
         <v>620</v>
       </c>
       <c r="D20" s="19" t="n">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="E20" s="19" t="n">
         <v>69</v>
@@ -7982,7 +7995,7 @@
         <v>663</v>
       </c>
       <c r="D35" s="19" t="n">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="E35" s="19" t="n">
         <v>10</v>
@@ -8002,10 +8015,10 @@
         <v>666</v>
       </c>
       <c r="D36" s="19" t="n">
-        <v>564</v>
+        <v>593</v>
       </c>
       <c r="E36" s="19" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F36" s="19" t="s">
         <v>667</v>
@@ -8265,7 +8278,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E145"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -9243,7 +9256,7 @@
         <v>851</v>
       </c>
       <c r="E59" s="19" t="s">
-        <v>646</v>
+        <v>852</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9254,13 +9267,13 @@
         <v>826</v>
       </c>
       <c r="C60" s="19" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="D60" s="19" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="E60" s="19" t="s">
-        <v>854</v>
+        <v>646</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9418,27 +9431,27 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="19" t="s">
+        <v>821</v>
+      </c>
+      <c r="B70" s="19" t="s">
+        <v>826</v>
+      </c>
+      <c r="C70" s="19" t="s">
         <v>882</v>
       </c>
-      <c r="B70" s="19" t="s">
+      <c r="D70" s="19" t="s">
         <v>883</v>
       </c>
-      <c r="C70" s="19" t="s">
+      <c r="E70" s="19" t="s">
         <v>884</v>
-      </c>
-      <c r="D70" s="19" t="s">
-        <v>885</v>
-      </c>
-      <c r="E70" s="19" t="s">
-        <v>886</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B71" s="19" t="s">
-        <v>883</v>
+        <v>886</v>
       </c>
       <c r="C71" s="19" t="s">
         <v>887</v>
@@ -9452,74 +9465,74 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B72" s="19" t="s">
-        <v>883</v>
+        <v>886</v>
       </c>
       <c r="C72" s="19" t="s">
         <v>890</v>
       </c>
-      <c r="D72" s="19"/>
+      <c r="D72" s="19" t="s">
+        <v>891</v>
+      </c>
       <c r="E72" s="19" t="s">
-        <v>889</v>
+        <v>892</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B73" s="19" t="s">
-        <v>883</v>
+        <v>886</v>
       </c>
       <c r="C73" s="19" t="s">
-        <v>891</v>
-      </c>
-      <c r="D73" s="19" t="s">
+        <v>893</v>
+      </c>
+      <c r="D73" s="19"/>
+      <c r="E73" s="19" t="s">
         <v>892</v>
-      </c>
-      <c r="E73" s="19" t="s">
-        <v>893</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B74" s="19" t="s">
-        <v>883</v>
+        <v>886</v>
       </c>
       <c r="C74" s="19" t="s">
         <v>894</v>
       </c>
-      <c r="D74" s="19"/>
+      <c r="D74" s="19" t="s">
+        <v>895</v>
+      </c>
       <c r="E74" s="19" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B75" s="19" t="s">
-        <v>883</v>
+        <v>886</v>
       </c>
       <c r="C75" s="19" t="s">
-        <v>896</v>
-      </c>
-      <c r="D75" s="19" t="s">
         <v>897</v>
       </c>
+      <c r="D75" s="19"/>
       <c r="E75" s="19" t="s">
         <v>898</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B76" s="19" t="s">
-        <v>883</v>
+        <v>886</v>
       </c>
       <c r="C76" s="19" t="s">
         <v>899</v>
@@ -9533,27 +9546,27 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B77" s="19" t="s">
+        <v>886</v>
+      </c>
+      <c r="C77" s="19" t="s">
         <v>902</v>
       </c>
-      <c r="C77" s="19" t="s">
+      <c r="D77" s="19" t="s">
         <v>903</v>
       </c>
-      <c r="D77" s="19" t="s">
+      <c r="E77" s="19" t="s">
         <v>904</v>
-      </c>
-      <c r="E77" s="19" t="s">
-        <v>905</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B78" s="19" t="s">
-        <v>902</v>
+        <v>905</v>
       </c>
       <c r="C78" s="19" t="s">
         <v>906</v>
@@ -9562,32 +9575,32 @@
         <v>907</v>
       </c>
       <c r="E78" s="19" t="s">
-        <v>843</v>
+        <v>908</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B79" s="19" t="s">
-        <v>902</v>
+        <v>905</v>
       </c>
       <c r="C79" s="19" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="D79" s="19" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="E79" s="19" t="s">
-        <v>910</v>
+        <v>843</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B80" s="19" t="s">
-        <v>902</v>
+        <v>905</v>
       </c>
       <c r="C80" s="19" t="s">
         <v>911</v>
@@ -9601,10 +9614,10 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B81" s="19" t="s">
-        <v>902</v>
+        <v>905</v>
       </c>
       <c r="C81" s="19" t="s">
         <v>914</v>
@@ -9618,10 +9631,10 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B82" s="19" t="s">
-        <v>902</v>
+        <v>905</v>
       </c>
       <c r="C82" s="19" t="s">
         <v>917</v>
@@ -9635,10 +9648,10 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B83" s="19" t="s">
-        <v>902</v>
+        <v>905</v>
       </c>
       <c r="C83" s="19" t="s">
         <v>920</v>
@@ -9652,10 +9665,10 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="19" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B84" s="19" t="s">
-        <v>902</v>
+        <v>905</v>
       </c>
       <c r="C84" s="19" t="s">
         <v>923</v>
@@ -9669,266 +9682,266 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="19" t="s">
+        <v>885</v>
+      </c>
+      <c r="B85" s="19" t="s">
+        <v>905</v>
+      </c>
+      <c r="C85" s="19" t="s">
         <v>926</v>
       </c>
-      <c r="B85" s="19" t="s">
+      <c r="D85" s="19" t="s">
         <v>927</v>
       </c>
-      <c r="C85" s="19" t="s">
+      <c r="E85" s="19" t="s">
         <v>928</v>
-      </c>
-      <c r="D85" s="19" t="s">
-        <v>929</v>
-      </c>
-      <c r="E85" s="19" t="s">
-        <v>930</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B86" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C86" s="19" t="s">
         <v>931</v>
       </c>
-      <c r="D86" s="19"/>
+      <c r="D86" s="19" t="s">
+        <v>932</v>
+      </c>
       <c r="E86" s="19" t="s">
-        <v>930</v>
+        <v>933</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B87" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C87" s="19" t="s">
-        <v>932</v>
-      </c>
-      <c r="D87" s="19" t="s">
+        <v>934</v>
+      </c>
+      <c r="D87" s="19"/>
+      <c r="E87" s="19" t="s">
         <v>933</v>
-      </c>
-      <c r="E87" s="19" t="s">
-        <v>930</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B88" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C88" s="19" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="D88" s="19" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="E88" s="19" t="s">
-        <v>788</v>
+        <v>933</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B89" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C89" s="19" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="D89" s="19" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="E89" s="19" t="s">
-        <v>794</v>
+        <v>788</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B90" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C90" s="19" t="s">
-        <v>938</v>
-      </c>
-      <c r="D90" s="19"/>
+        <v>939</v>
+      </c>
+      <c r="D90" s="19" t="s">
+        <v>940</v>
+      </c>
       <c r="E90" s="19" t="s">
         <v>794</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B91" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C91" s="19" t="s">
-        <v>939</v>
+        <v>941</v>
       </c>
       <c r="D91" s="19"/>
       <c r="E91" s="19" t="s">
-        <v>930</v>
+        <v>794</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B92" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C92" s="19" t="s">
-        <v>940</v>
+        <v>942</v>
       </c>
       <c r="D92" s="19"/>
       <c r="E92" s="19" t="s">
-        <v>930</v>
+        <v>933</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B93" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C93" s="19" t="s">
-        <v>941</v>
-      </c>
-      <c r="D93" s="19" t="s">
-        <v>942</v>
-      </c>
+        <v>943</v>
+      </c>
+      <c r="D93" s="19"/>
       <c r="E93" s="19" t="s">
-        <v>930</v>
+        <v>933</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B94" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C94" s="19" t="s">
-        <v>943</v>
-      </c>
-      <c r="D94" s="19"/>
+        <v>944</v>
+      </c>
+      <c r="D94" s="19" t="s">
+        <v>945</v>
+      </c>
       <c r="E94" s="19" t="s">
-        <v>587</v>
+        <v>933</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B95" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C95" s="19" t="s">
-        <v>944</v>
-      </c>
-      <c r="D95" s="19" t="s">
-        <v>945</v>
-      </c>
+        <v>946</v>
+      </c>
+      <c r="D95" s="19"/>
       <c r="E95" s="19" t="s">
-        <v>930</v>
+        <v>587</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B96" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C96" s="19" t="s">
-        <v>946</v>
-      </c>
-      <c r="D96" s="19"/>
+        <v>947</v>
+      </c>
+      <c r="D96" s="19" t="s">
+        <v>948</v>
+      </c>
       <c r="E96" s="19" t="s">
-        <v>930</v>
+        <v>933</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B97" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C97" s="19" t="s">
-        <v>947</v>
+        <v>949</v>
       </c>
       <c r="D97" s="19"/>
       <c r="E97" s="19" t="s">
-        <v>930</v>
+        <v>933</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B98" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C98" s="19" t="s">
-        <v>948</v>
-      </c>
-      <c r="D98" s="19" t="s">
-        <v>949</v>
-      </c>
+        <v>950</v>
+      </c>
+      <c r="D98" s="19"/>
       <c r="E98" s="19" t="s">
-        <v>784</v>
+        <v>933</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B99" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C99" s="19" t="s">
-        <v>950</v>
-      </c>
-      <c r="D99" s="19"/>
+        <v>951</v>
+      </c>
+      <c r="D99" s="19" t="s">
+        <v>952</v>
+      </c>
       <c r="E99" s="19" t="s">
         <v>784</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B100" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C100" s="19" t="s">
-        <v>951</v>
-      </c>
-      <c r="D100" s="19" t="s">
-        <v>952</v>
-      </c>
+        <v>953</v>
+      </c>
+      <c r="D100" s="19"/>
       <c r="E100" s="19" t="s">
-        <v>953</v>
+        <v>784</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B101" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C101" s="19" t="s">
         <v>954</v>
@@ -9937,21 +9950,21 @@
         <v>955</v>
       </c>
       <c r="E101" s="19" t="s">
-        <v>587</v>
+        <v>956</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B102" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C102" s="19" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="D102" s="19" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="E102" s="19" t="s">
         <v>587</v>
@@ -9959,89 +9972,89 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B103" s="19" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="C103" s="19" t="s">
-        <v>958</v>
-      </c>
-      <c r="D103" s="19"/>
+        <v>959</v>
+      </c>
+      <c r="D103" s="19" t="s">
+        <v>960</v>
+      </c>
       <c r="E103" s="19" t="s">
-        <v>930</v>
+        <v>587</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B104" s="19" t="s">
-        <v>959</v>
+        <v>930</v>
       </c>
       <c r="C104" s="19" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="D104" s="19"/>
       <c r="E104" s="19" t="s">
-        <v>961</v>
+        <v>933</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B105" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="C105" s="19" t="s">
-        <v>962</v>
-      </c>
-      <c r="D105" s="19" t="s">
         <v>963</v>
       </c>
+      <c r="D105" s="19"/>
       <c r="E105" s="19" t="s">
-        <v>930</v>
+        <v>964</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B106" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="C106" s="19" t="s">
-        <v>964</v>
-      </c>
-      <c r="D106" s="19"/>
+        <v>965</v>
+      </c>
+      <c r="D106" s="19" t="s">
+        <v>966</v>
+      </c>
       <c r="E106" s="19" t="s">
-        <v>930</v>
-      </c>
-    </row>
-    <row r="107" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B107" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="C107" s="19" t="s">
-        <v>965</v>
-      </c>
-      <c r="D107" s="19" t="s">
-        <v>966</v>
-      </c>
+        <v>967</v>
+      </c>
+      <c r="D107" s="19"/>
       <c r="E107" s="19" t="s">
-        <v>967</v>
+        <v>933</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B108" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="C108" s="19" t="s">
         <v>968</v>
@@ -10050,166 +10063,166 @@
         <v>969</v>
       </c>
       <c r="E108" s="19" t="s">
-        <v>967</v>
-      </c>
-    </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B109" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="C109" s="19" t="s">
+        <v>971</v>
+      </c>
+      <c r="D109" s="19" t="s">
+        <v>972</v>
+      </c>
+      <c r="E109" s="19" t="s">
         <v>970</v>
       </c>
-      <c r="D109" s="19" t="s">
-        <v>971</v>
-      </c>
-      <c r="E109" s="19" t="s">
-        <v>972</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B110" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="C110" s="19" t="s">
         <v>973</v>
       </c>
-      <c r="D110" s="19"/>
+      <c r="D110" s="19" t="s">
+        <v>974</v>
+      </c>
       <c r="E110" s="19" t="s">
-        <v>961</v>
-      </c>
-    </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B111" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="C111" s="19" t="s">
-        <v>974</v>
-      </c>
-      <c r="D111" s="19" t="s">
-        <v>975</v>
-      </c>
+        <v>976</v>
+      </c>
+      <c r="D111" s="19"/>
       <c r="E111" s="19" t="s">
-        <v>930</v>
-      </c>
-    </row>
-    <row r="112" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B112" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="C112" s="19" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="D112" s="19" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="E112" s="19" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="19" t="s">
+        <v>929</v>
+      </c>
+      <c r="B113" s="19" t="s">
+        <v>962</v>
+      </c>
+      <c r="C113" s="19" t="s">
+        <v>979</v>
+      </c>
+      <c r="D113" s="19" t="s">
+        <v>980</v>
+      </c>
+      <c r="E113" s="19" t="s">
         <v>846</v>
-      </c>
-    </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="19" t="s">
-        <v>926</v>
-      </c>
-      <c r="B113" s="19" t="s">
-        <v>959</v>
-      </c>
-      <c r="C113" s="19" t="s">
-        <v>978</v>
-      </c>
-      <c r="D113" s="19" t="s">
-        <v>979</v>
-      </c>
-      <c r="E113" s="19" t="s">
-        <v>881</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B114" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="C114" s="19" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="D114" s="19" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="E114" s="19" t="s">
-        <v>655</v>
+        <v>884</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B115" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="C115" s="19" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="D115" s="19" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="E115" s="19" t="s">
-        <v>930</v>
+        <v>655</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="19" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="B116" s="19" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="C116" s="19" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="D116" s="19" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="E116" s="19" t="s">
-        <v>655</v>
+        <v>933</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="19" t="s">
-        <v>986</v>
+        <v>929</v>
       </c>
       <c r="B117" s="19" t="s">
+        <v>962</v>
+      </c>
+      <c r="C117" s="19" t="s">
         <v>987</v>
       </c>
-      <c r="C117" s="19" t="s">
+      <c r="D117" s="19" t="s">
         <v>988</v>
       </c>
-      <c r="D117" s="19" t="s">
-        <v>989</v>
-      </c>
       <c r="E117" s="19" t="s">
-        <v>990</v>
+        <v>655</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="19" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="B118" s="19" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="C118" s="19" t="s">
         <v>991</v>
@@ -10223,10 +10236,10 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="19" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="B119" s="19" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="C119" s="19" t="s">
         <v>994</v>
@@ -10235,245 +10248,245 @@
         <v>995</v>
       </c>
       <c r="E119" s="19" t="s">
-        <v>881</v>
+        <v>996</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="19" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="B120" s="19" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="C120" s="19" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="D120" s="19" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="E120" s="19" t="s">
-        <v>961</v>
+        <v>884</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="19" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="B121" s="19" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="C121" s="19" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="D121" s="19" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="E121" s="19" t="s">
-        <v>961</v>
+        <v>964</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="19" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="B122" s="19" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="C122" s="19" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="D122" s="19" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="E122" s="19" t="s">
-        <v>990</v>
+        <v>964</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="19" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="B123" s="19" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="C123" s="19" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="D123" s="19" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="E123" s="19" t="s">
-        <v>889</v>
+        <v>993</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="19" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="B124" s="19" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="C124" s="19" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="D124" s="19" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="E124" s="19" t="s">
-        <v>1006</v>
-      </c>
-    </row>
-    <row r="125" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="19" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="B125" s="19" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="C125" s="19" t="s">
         <v>1007</v>
       </c>
-      <c r="D125" s="19"/>
+      <c r="D125" s="19" t="s">
+        <v>1008</v>
+      </c>
       <c r="E125" s="19" t="s">
-        <v>1008</v>
-      </c>
-    </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="19" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="B126" s="19" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="C126" s="19" t="s">
-        <v>1009</v>
-      </c>
-      <c r="D126" s="19" t="s">
         <v>1010</v>
       </c>
+      <c r="D126" s="19"/>
       <c r="E126" s="19" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="19" t="s">
+        <v>989</v>
+      </c>
+      <c r="B127" s="19" t="s">
+        <v>990</v>
+      </c>
+      <c r="C127" s="19" t="s">
+        <v>1012</v>
+      </c>
+      <c r="D127" s="19" t="s">
+        <v>1013</v>
+      </c>
+      <c r="E127" s="19" t="s">
         <v>655</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A127" s="19" t="s">
-        <v>986</v>
-      </c>
-      <c r="B127" s="19" t="s">
-        <v>987</v>
-      </c>
-      <c r="C127" s="19" t="s">
+    <row r="128" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="19" t="s">
+        <v>989</v>
+      </c>
+      <c r="B128" s="19" t="s">
+        <v>990</v>
+      </c>
+      <c r="C128" s="19" t="s">
+        <v>1014</v>
+      </c>
+      <c r="D128" s="19"/>
+      <c r="E128" s="19" t="s">
         <v>1011</v>
-      </c>
-      <c r="D127" s="19"/>
-      <c r="E127" s="19" t="s">
-        <v>1008</v>
-      </c>
-    </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A128" s="19" t="s">
-        <v>986</v>
-      </c>
-      <c r="B128" s="19" t="s">
-        <v>987</v>
-      </c>
-      <c r="C128" s="19" t="s">
-        <v>1012</v>
-      </c>
-      <c r="D128" s="19" t="s">
-        <v>1013</v>
-      </c>
-      <c r="E128" s="19" t="s">
-        <v>655</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="19" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="B129" s="19" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="C129" s="19" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="D129" s="19" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="E129" s="19" t="s">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="130" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="19" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="B130" s="19" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="C130" s="19" t="s">
         <v>1017</v>
       </c>
-      <c r="D130" s="19"/>
+      <c r="D130" s="19" t="s">
+        <v>1018</v>
+      </c>
       <c r="E130" s="19" t="s">
-        <v>1008</v>
-      </c>
-    </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="19" t="s">
-        <v>1018</v>
+        <v>989</v>
       </c>
       <c r="B131" s="19" t="s">
-        <v>1019</v>
+        <v>990</v>
       </c>
       <c r="C131" s="19" t="s">
         <v>1020</v>
       </c>
       <c r="D131" s="19"/>
       <c r="E131" s="19" t="s">
-        <v>1021</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B132" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C132" s="19" t="s">
-        <v>1022</v>
-      </c>
-      <c r="D132" s="19" t="s">
         <v>1023</v>
       </c>
+      <c r="D132" s="19"/>
       <c r="E132" s="19" t="s">
-        <v>846</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B133" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C133" s="19" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="D133" s="19" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="E133" s="19" t="s">
-        <v>1026</v>
+        <v>846</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B134" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C134" s="19" t="s">
         <v>1027</v>
@@ -10487,10 +10500,10 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B135" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C135" s="19" t="s">
         <v>1030</v>
@@ -10499,169 +10512,186 @@
         <v>1031</v>
       </c>
       <c r="E135" s="19" t="s">
-        <v>1021</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B136" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C136" s="19" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="D136" s="19" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="E136" s="19" t="s">
-        <v>846</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B137" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C137" s="19" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="D137" s="19" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="E137" s="19" t="s">
-        <v>881</v>
+        <v>846</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B138" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C138" s="19" t="s">
-        <v>1036</v>
-      </c>
-      <c r="D138" s="19"/>
+        <v>1037</v>
+      </c>
+      <c r="D138" s="19" t="s">
+        <v>1038</v>
+      </c>
       <c r="E138" s="19" t="s">
-        <v>846</v>
+        <v>884</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B139" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C139" s="19" t="s">
-        <v>1037</v>
-      </c>
-      <c r="D139" s="19" t="s">
-        <v>1038</v>
-      </c>
+        <v>1039</v>
+      </c>
+      <c r="D139" s="19"/>
       <c r="E139" s="19" t="s">
         <v>846</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B140" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C140" s="19" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="D140" s="19" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="E140" s="19" t="s">
-        <v>967</v>
+        <v>846</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B141" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C141" s="19" t="s">
-        <v>1041</v>
-      </c>
-      <c r="D141" s="19"/>
+        <v>1042</v>
+      </c>
+      <c r="D141" s="19" t="s">
+        <v>1043</v>
+      </c>
       <c r="E141" s="19" t="s">
-        <v>1021</v>
+        <v>970</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B142" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C142" s="19" t="s">
-        <v>1042</v>
+        <v>1044</v>
       </c>
       <c r="D142" s="19"/>
       <c r="E142" s="19" t="s">
-        <v>1021</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B143" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C143" s="19" t="s">
-        <v>1043</v>
+        <v>1045</v>
       </c>
       <c r="D143" s="19"/>
       <c r="E143" s="19" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B144" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C144" s="19" t="s">
-        <v>1044</v>
+        <v>1046</v>
       </c>
       <c r="D144" s="19"/>
       <c r="E144" s="19" t="s">
-        <v>1021</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="19" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
       <c r="B145" s="19" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="C145" s="19" t="s">
-        <v>1045</v>
+        <v>1047</v>
       </c>
       <c r="D145" s="19"/>
       <c r="E145" s="19" t="s">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="19" t="s">
         <v>1021</v>
       </c>
+      <c r="B146" s="19" t="s">
+        <v>1022</v>
+      </c>
+      <c r="C146" s="19" t="s">
+        <v>1048</v>
+      </c>
+      <c r="D146" s="19"/>
+      <c r="E146" s="19" t="s">
+        <v>1024</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E145"/>
+  <autoFilter ref="A1:E146"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
VISU PTBG 1.0.0 : classeur des versions et dépendances (REQ 3004)
Nouveau docs/recapitulatif/Dependances_versions_VISU_PTBG.xlsx, en réponse
au commentaire de relecture sur REQ 3004 (paquets transverses ou restrictifs,
sensibilité à la version de Python, à l'OS et au 32/64 bits) : bibliothèques
(figées / poste Spyder), arbre des dépendances avec contraintes vérifiées,
sensibilités, bibliothèque standard, campagnes de tests, impact d'une montée
de version, procédure et relevé des postes à remplir.

Versions du poste Windows 11 / Spyder 6 (numpy 2.2.0, matplotlib 3.9.3…)
vérifiées : 145 tests OK ; consignées dans DEPENDANCES.md et COMPATIBILITE_OS.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xr679nCBrcWe6H8towhecz
</commit_message>
<xml_diff>
--- a/docs/recapitulatif/Recapitulatif_requis_VISU_PTBG.xlsx
+++ b/docs/recapitulatif/Recapitulatif_requis_VISU_PTBG.xlsx
@@ -704,7 +704,7 @@
     <t xml:space="preserve">Paquets documentés et alignés sur la version du noyau Python</t>
   </si>
   <si>
-    <t xml:space="preserve">requirements.txt figé et commenté, docs/DEPENDANCES.md (versions, licences, Python supportés, wheels, impacts de montée de version), relevé au démarrage</t>
+    <t xml:space="preserve">requirements.txt figé et commenté, docs/DEPENDANCES.md (versions, licences, Python supportés, wheels, impacts de montée de version) et classeur docs/recapitulatif/Dependances_versions_VISU_PTBG.xlsx (dépendances, sensibilités Python / OS / 32-64 bits, campagnes, relevé des postes), relevé au démarrage</t>
   </si>
   <si>
     <t xml:space="preserve">system/environment.py, requirements.txt</t>
@@ -1548,10 +1548,10 @@
     <t xml:space="preserve">Il y a des packages transverses toute version et d’autre plus restrictifs avec independances. Le plus fréquemment il y a une sensibilité à la version de python, l’OS, et le cœur 32 ou 63 bits</t>
   </si>
   <si>
-    <t xml:space="preserve">Sensibilités relevées par Sébastien traitées : versions figées dans requirements.txt (identiques Python 3.11 à 3.14, Windows et SLES) ; DEPENDANCES.md donne pour chaque paquet la version, le type (direct / transitif), les Python supportés, les wheels win_amd64 / manylinux, la licence, et distingue les composants compilés (sensibles à Python, à l'OS et au 32/64 bits : numpy, matplotlib, contourpy, kiwisolver, pillow) du Python pur. Cible 64 bits uniquement. Relevé des versions au démarrage et outil d'audit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">requirements.txt ; docs/DEPENDANCES.md ; ptbg/system/environment.py ; tools/audit_environnement.py</t>
+    <t xml:space="preserve">Sensibilités relevées par Sébastien traitées : versions figées dans requirements.txt (identiques Python 3.11 à 3.14, Windows et SLES) ; DEPENDANCES.md donne pour chaque paquet la version, le type (direct / transitif), les Python supportés, les wheels win_amd64 / manylinux, la licence, et distingue les composants compilés (sensibles à Python, à l'OS et au 32/64 bits : numpy, matplotlib, contourpy, fonttools, kiwisolver, pillow) du Python pur. Cible 64 bits uniquement. Relevé des versions au démarrage et outil d'audit. Classeur dédié docs/recapitulatif/Dependances_versions_VISU_PTBG.xlsx (bibliothèques, dépendances, sensibilités, campagnes de tests, impact d'une montée de version, relevé des postes).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">requirements.txt ; docs/DEPENDANCES.md ; docs/recapitulatif/Dependances_versions_VISU_PTBG.xlsx ; ptbg/system/environment.py ; tools/audit_environnement.py</t>
   </si>
   <si>
     <t xml:space="preserve">test_architecture.test_third_party_libraries_are_documented_and_pinned</t>
@@ -6884,7 +6884,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
         <v>209</v>
       </c>

</xml_diff>